<commit_message>
Edit AC + DCT Logic
</commit_message>
<xml_diff>
--- a/FCIS_HCI/Task2/Feature_Map.xlsx
+++ b/FCIS_HCI/Task2/Feature_Map.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM3"/>
+  <dimension ref="A1:DO3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,7 +544,247 @@
       <c r="AL1" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="AX1" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="AY1" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="AZ1" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="BA1" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="BB1" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="BC1" s="1" t="n">
+        <v>54</v>
+      </c>
+      <c r="BD1" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="BE1" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="BF1" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="BG1" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="BH1" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="BI1" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="BJ1" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="BK1" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="BL1" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="BN1" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="BO1" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="BP1" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="BQ1" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="BR1" s="1" t="n">
+        <v>69</v>
+      </c>
+      <c r="BS1" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="BT1" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="BU1" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="BV1" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="BW1" s="1" t="n">
+        <v>74</v>
+      </c>
+      <c r="BX1" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="BY1" s="1" t="n">
+        <v>76</v>
+      </c>
+      <c r="BZ1" s="1" t="n">
+        <v>77</v>
+      </c>
+      <c r="CA1" s="1" t="n">
+        <v>78</v>
+      </c>
+      <c r="CB1" s="1" t="n">
+        <v>79</v>
+      </c>
+      <c r="CC1" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="CD1" s="1" t="n">
+        <v>81</v>
+      </c>
+      <c r="CE1" s="1" t="n">
+        <v>82</v>
+      </c>
+      <c r="CF1" s="1" t="n">
+        <v>83</v>
+      </c>
+      <c r="CG1" s="1" t="n">
+        <v>84</v>
+      </c>
+      <c r="CH1" s="1" t="n">
+        <v>85</v>
+      </c>
+      <c r="CI1" s="1" t="n">
+        <v>86</v>
+      </c>
+      <c r="CJ1" s="1" t="n">
+        <v>87</v>
+      </c>
+      <c r="CK1" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="CL1" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="CM1" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="CN1" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="CO1" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="CP1" s="1" t="n">
+        <v>93</v>
+      </c>
+      <c r="CQ1" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="CR1" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="CS1" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="CT1" s="1" t="n">
+        <v>97</v>
+      </c>
+      <c r="CU1" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="CV1" s="1" t="n">
+        <v>99</v>
+      </c>
+      <c r="CW1" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="CX1" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="CY1" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="CZ1" s="1" t="n">
+        <v>103</v>
+      </c>
+      <c r="DA1" s="1" t="n">
+        <v>104</v>
+      </c>
+      <c r="DB1" s="1" t="n">
+        <v>105</v>
+      </c>
+      <c r="DC1" s="1" t="n">
+        <v>106</v>
+      </c>
+      <c r="DD1" s="1" t="n">
+        <v>107</v>
+      </c>
+      <c r="DE1" s="1" t="n">
+        <v>108</v>
+      </c>
+      <c r="DF1" s="1" t="n">
+        <v>109</v>
+      </c>
+      <c r="DG1" s="1" t="n">
+        <v>110</v>
+      </c>
+      <c r="DH1" s="1" t="n">
+        <v>111</v>
+      </c>
+      <c r="DI1" s="1" t="n">
+        <v>112</v>
+      </c>
+      <c r="DJ1" s="1" t="n">
+        <v>113</v>
+      </c>
+      <c r="DK1" s="1" t="n">
+        <v>114</v>
+      </c>
+      <c r="DL1" s="1" t="n">
+        <v>115</v>
+      </c>
+      <c r="DM1" s="1" t="n">
+        <v>116</v>
+      </c>
+      <c r="DN1" s="1" t="n">
+        <v>117</v>
+      </c>
+      <c r="DO1" s="1" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
@@ -606,66 +846,306 @@
         <v>6185070.58289999</v>
       </c>
       <c r="S2" t="n">
-        <v>16515947.26197905</v>
+        <v>1.561272068394008</v>
       </c>
       <c r="T2" t="n">
-        <v>23356798.14790668</v>
+        <v>8.765014528609948</v>
       </c>
       <c r="U2" t="n">
-        <v>23357283.93063478</v>
+        <v>1.350915440702132</v>
       </c>
       <c r="V2" t="n">
-        <v>23357213.51693717</v>
+        <v>7.853872586316713</v>
       </c>
       <c r="W2" t="n">
-        <v>23357906.12848926</v>
+        <v>11.41097191401333</v>
       </c>
       <c r="X2" t="n">
-        <v>23358044.66966552</v>
+        <v>6.002398453679779</v>
       </c>
       <c r="Y2" t="n">
-        <v>23358943.60984568</v>
+        <v>5.307213312576595</v>
       </c>
       <c r="Z2" t="n">
-        <v>23359292.40602936</v>
+        <v>10.25684553057132</v>
       </c>
       <c r="AA2" t="n">
-        <v>23360397.12740724</v>
+        <v>6.828034016986832</v>
       </c>
       <c r="AB2" t="n">
-        <v>23360957.86746119</v>
+        <v>3.695059563052363</v>
       </c>
       <c r="AC2" t="n">
-        <v>23362267.66329943</v>
+        <v>4.427175443153377</v>
       </c>
       <c r="AD2" t="n">
-        <v>23363042.74196035</v>
+        <v>4.78093453059839</v>
       </c>
       <c r="AE2" t="n">
-        <v>23364556.71008626</v>
+        <v>4.093646342002993</v>
       </c>
       <c r="AF2" t="n">
-        <v>23365548.95754114</v>
+        <v>4.156747255218278</v>
       </c>
       <c r="AG2" t="n">
-        <v>23367265.85320877</v>
+        <v>4.059769360876548</v>
       </c>
       <c r="AH2" t="n">
-        <v>23368478.95377436</v>
+        <v>3.33193368918666</v>
       </c>
       <c r="AI2" t="n">
-        <v>23370396.73951993</v>
+        <v>2.907886217411541</v>
       </c>
       <c r="AJ2" t="n">
-        <v>23371836.20979403</v>
+        <v>2.795023102032286</v>
       </c>
       <c r="AK2" t="n">
-        <v>23373953.13742056</v>
+        <v>2.423646106264151</v>
       </c>
       <c r="AL2" t="n">
-        <v>23375623.97616179</v>
-      </c>
-      <c r="AM2" t="inlineStr">
+        <v>2.030746404556313</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>1.755127459875706</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>1.555737073357487</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>1.255128719089491</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0.9486641353464047</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0.6571371827312422</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0.4164127719521873</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0.2449107973370891</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>0.147633306045193</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>0.03985123274027111</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>-0.06574323668558787</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>-0.1558163363465062</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>-0.1922736775066616</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>-0.2037877624524587</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>-0.19350122883926</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>-0.1864913245587149</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>-0.1724971198042735</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>-0.1636479913025797</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>-0.1486552090956218</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>-0.139543674578662</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>-0.1264732524009388</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>-0.1193458612609486</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>-0.1086576958539843</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>-0.1031808258277369</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>-0.0943785871541737</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>-0.09015586991369062</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>-0.08281127099694932</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>-0.0794951353614365</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>-0.07326064089063232</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>-0.07060119003161588</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>-0.06523318327263308</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>-0.06306277033428442</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>-0.05838904967365953</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>-0.05659155683385717</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>-0.05248413153967209</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>-0.05097484365597936</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>-0.04733667337647207</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>-0.04605297823389293</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>-0.0428088586186139</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>-0.04170349073503533</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>-0.03879386018815635</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>-0.03783041212207141</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>-0.03520743323002493</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>-0.03435743476362371</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>-0.03198214463080897</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>-0.03122301416748653</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>-0.02906327147552126</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>-0.02837684673354068</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>-0.02640589824245733</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>-0.025777411648639</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>-0.02397276333630019</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>-0.02339005960338385</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>-0.02173264679532758</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>-0.02118561035295706</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>-0.01965915050786253</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>-0.01913926540265451</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>-0.01772975530281173</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>-0.01722976984365832</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>-0.01592508581714785</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>-0.01543874870614048</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>-0.01422832946170627</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>-0.01375018287972696</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>-0.01262477218729696</v>
+      </c>
+      <c r="CW2" t="n">
+        <v>-0.01214998581274318</v>
+      </c>
+      <c r="CX2" t="n">
+        <v>-0.01110142343300757</v>
+      </c>
+      <c r="CY2" t="n">
+        <v>-0.01062566023873179</v>
+      </c>
+      <c r="CZ2" t="n">
+        <v>-0.009646709539926634</v>
+      </c>
+      <c r="DA2" t="n">
+        <v>-0.00916601547069984</v>
+      </c>
+      <c r="DB2" t="n">
+        <v>-0.008250220449825818</v>
+      </c>
+      <c r="DC2" t="n">
+        <v>-0.007760932482886229</v>
+      </c>
+      <c r="DD2" t="n">
+        <v>-0.006902497733612734</v>
+      </c>
+      <c r="DE2" t="n">
+        <v>-0.006401165798485042</v>
+      </c>
+      <c r="DF2" t="n">
+        <v>-0.005594854817370987</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>-0.005078174247709288</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>-0.004319222258521549</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>-0.003783974003207735</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>-0.003068012280590171</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>-0.00251100866544629</v>
+      </c>
+      <c r="DL2" t="n">
+        <v>-0.001833997882518368</v>
+      </c>
+      <c r="DM2" t="n">
+        <v>-0.001252032051763718</v>
+      </c>
+      <c r="DN2" t="n">
+        <v>-0.0006102025841769887</v>
+      </c>
+      <c r="DO2" t="inlineStr">
         <is>
           <t>Ali</t>
         </is>
@@ -727,66 +1207,306 @@
         <v>2508303.042170639</v>
       </c>
       <c r="S3" t="n">
-        <v>8713134.599703075</v>
+        <v>-1.138046985875017</v>
       </c>
       <c r="T3" t="n">
-        <v>12213017.03520529</v>
+        <v>11.42831392572541</v>
       </c>
       <c r="U3" t="n">
-        <v>12322303.03030368</v>
+        <v>2.234944315678328</v>
       </c>
       <c r="V3" t="n">
-        <v>12213218.399378</v>
+        <v>3.12051106045639</v>
       </c>
       <c r="W3" t="n">
-        <v>12322512.66969361</v>
+        <v>10.63693226854349</v>
       </c>
       <c r="X3" t="n">
-        <v>12213622.05011246</v>
+        <v>9.960850230424183</v>
       </c>
       <c r="Y3" t="n">
-        <v>12322863.23683178</v>
+        <v>4.688907082865189</v>
       </c>
       <c r="Z3" t="n">
-        <v>12214229.17514465</v>
+        <v>6.271002194578324</v>
       </c>
       <c r="AA3" t="n">
-        <v>12323356.3017709</v>
+        <v>5.750320601976259</v>
       </c>
       <c r="AB3" t="n">
-        <v>12215041.88846916</v>
+        <v>5.075794359208995</v>
       </c>
       <c r="AC3" t="n">
-        <v>12323994.00725464</v>
+        <v>5.018076007587888</v>
       </c>
       <c r="AD3" t="n">
-        <v>12216063.08401798</v>
+        <v>5.701170058990931</v>
       </c>
       <c r="AE3" t="n">
-        <v>12324779.40764321</v>
+        <v>4.997788777055418</v>
       </c>
       <c r="AF3" t="n">
-        <v>12217296.11768754</v>
+        <v>4.354922540410181</v>
       </c>
       <c r="AG3" t="n">
-        <v>12325716.16966465</v>
+        <v>4.356963184980231</v>
       </c>
       <c r="AH3" t="n">
-        <v>12218745.2268156</v>
+        <v>4.422704975723772</v>
       </c>
       <c r="AI3" t="n">
-        <v>12326808.30034945</v>
+        <v>3.676306599379933</v>
       </c>
       <c r="AJ3" t="n">
-        <v>12220415.13327163</v>
+        <v>2.898954205495314</v>
       </c>
       <c r="AK3" t="n">
-        <v>12328060.23938321</v>
+        <v>2.368803417593357</v>
       </c>
       <c r="AL3" t="n">
-        <v>12222312.15622997</v>
-      </c>
-      <c r="AM3" t="inlineStr">
+        <v>2.145459708957774</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>1.874838737163905</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>1.564299479945462</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>1.141006273006712</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>0.7449786827596542</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0.3800858166978826</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>0.1863228209874065</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0.05329461073795287</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>-0.02339702822889887</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>-0.1204307896457193</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>-0.1640904350576735</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>-0.1985603702502647</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>-0.1955975491617729</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>-0.2044277227812163</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>-0.1870195806234984</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>-0.1828858335173345</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>-0.161117523093517</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>-0.1565154898146995</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>-0.1382869684538059</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>-0.1352980764093465</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>-0.1195229441754138</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>-0.1170588779450046</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>-0.1034264720259944</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>-0.1018855691673199</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>-0.0903133657409545</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>-0.08951329382616879</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>-0.07955951867251093</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>-0.07923047571045339</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>-0.07056660489803659</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>-0.07056096679721617</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>-0.06295918192594466</v>
+      </c>
+      <c r="BQ3" t="n">
+        <v>-0.06316992981080811</v>
+      </c>
+      <c r="BR3" t="n">
+        <v>-0.05644504020941438</v>
+      </c>
+      <c r="BS3" t="n">
+        <v>-0.05679309773316722</v>
+      </c>
+      <c r="BT3" t="n">
+        <v>-0.05080398970935857</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>-0.05123609619640932</v>
+      </c>
+      <c r="BV3" t="n">
+        <v>-0.04587224177573476</v>
+      </c>
+      <c r="BW3" t="n">
+        <v>-0.04635025667793785</v>
+      </c>
+      <c r="BX3" t="n">
+        <v>-0.04152353912183523</v>
+      </c>
+      <c r="BY3" t="n">
+        <v>-0.04202027886680201</v>
+      </c>
+      <c r="BZ3" t="n">
+        <v>-0.03765938040537942</v>
+      </c>
+      <c r="CA3" t="n">
+        <v>-0.03815509875164622</v>
+      </c>
+      <c r="CB3" t="n">
+        <v>-0.03420153442322746</v>
+      </c>
+      <c r="CC3" t="n">
+        <v>-0.03468180827008757</v>
+      </c>
+      <c r="CD3" t="n">
+        <v>-0.03108707947734529</v>
+      </c>
+      <c r="CE3" t="n">
+        <v>-0.03154121482524833</v>
+      </c>
+      <c r="CF3" t="n">
+        <v>-0.02826469528778032</v>
+      </c>
+      <c r="CG3" t="n">
+        <v>-0.02868472497716841</v>
+      </c>
+      <c r="CH3" t="n">
+        <v>-0.0256921105662236</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>-0.02607202211174044</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>-0.02333412585283447</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>-0.02366933507275391</v>
+      </c>
+      <c r="CL3" t="n">
+        <v>-0.0211611625904992</v>
+      </c>
+      <c r="CM3" t="n">
+        <v>-0.02144811943287615</v>
+      </c>
+      <c r="CN3" t="n">
+        <v>-0.01914814436726305</v>
+      </c>
+      <c r="CO3" t="n">
+        <v>-0.01938404038013407</v>
+      </c>
+      <c r="CP3" t="n">
+        <v>-0.01727362639881377</v>
+      </c>
+      <c r="CQ3" t="n">
+        <v>-0.01745617751169298</v>
+      </c>
+      <c r="CR3" t="n">
+        <v>-0.01551911781062698</v>
+      </c>
+      <c r="CS3" t="n">
+        <v>-0.01564639804260504</v>
+      </c>
+      <c r="CT3" t="n">
+        <v>-0.01386854147666594</v>
+      </c>
+      <c r="CU3" t="n">
+        <v>-0.01393885485883906</v>
+      </c>
+      <c r="CV3" t="n">
+        <v>-0.01230780155453171</v>
+      </c>
+      <c r="CW3" t="n">
+        <v>-0.01231958186985449</v>
+      </c>
+      <c r="CX3" t="n">
+        <v>-0.01082443282075984</v>
+      </c>
+      <c r="CY3" t="n">
+        <v>-0.01077616339912058</v>
+      </c>
+      <c r="CZ3" t="n">
+        <v>-0.009407313089780711</v>
+      </c>
+      <c r="DA3" t="n">
+        <v>-0.009297461331008172</v>
+      </c>
+      <c r="DB3" t="n">
+        <v>-0.008046424900147731</v>
+      </c>
+      <c r="DC3" t="n">
+        <v>-0.00787338729997078</v>
+      </c>
+      <c r="DD3" t="n">
+        <v>-0.006732655512073915</v>
+      </c>
+      <c r="DE3" t="n">
+        <v>-0.006494710077647348</v>
+      </c>
+      <c r="DF3" t="n">
+        <v>-0.005457626888755396</v>
+      </c>
+      <c r="DG3" t="n">
+        <v>-0.005152890464351856</v>
+      </c>
+      <c r="DH3" t="n">
+        <v>-0.004213549005619655</v>
+      </c>
+      <c r="DI3" t="n">
+        <v>-0.003839937528542059</v>
+      </c>
+      <c r="DJ3" t="n">
+        <v>-0.002993091159552819</v>
+      </c>
+      <c r="DK3" t="n">
+        <v>-0.002548281204378888</v>
+      </c>
+      <c r="DL3" t="n">
+        <v>-0.001789266911046195</v>
+      </c>
+      <c r="DM3" t="n">
+        <v>-0.001270657102490302</v>
+      </c>
+      <c r="DN3" t="n">
+        <v>-0.0005953289921194482</v>
+      </c>
+      <c r="DO3" t="inlineStr">
         <is>
           <t>Mohamed</t>
         </is>
@@ -815,52 +1535,52 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>28</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>29</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>30</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>31</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>32</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>33</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>34</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>35</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>36</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>37</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>